<commit_message>
Fix column alignment after inserting the Insider Flow column
Adding a column to the tier sheet header shifted every field to its
right, but three places wrote to fixed indices and were not moved with
it. The performance loop started at column 18, overwriting the
Conviction cell and pushing 1M through 1Y one column left of their
headers, so the workbook reported a conviction rating in the wrong place
and a wrong value under every performance heading. Column widths and the
conditional-formatting ranges were still keyed to the old layout too, so
the score colour scales were painting the wrong columns.

Verified by reading the saved workbook back and checking each field
against its own header rather than by position.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JddThw18de4GoJHnFCFNA6
</commit_message>
<xml_diff>
--- a/output/screener_output_20260908.xlsx
+++ b/output/screener_output_20260908.xlsx
@@ -14865,15 +14865,16 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -15108,19 +15109,24 @@
       <c r="Q5" s="39" t="n">
         <v>4.4</v>
       </c>
-      <c r="R5" s="34" t="n">
+      <c r="R5" s="23" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S5" s="34" t="n">
         <v>0.007246376799999999</v>
       </c>
-      <c r="S5" s="34" t="n">
+      <c r="T5" s="34" t="n">
         <v>-0.2553571</v>
       </c>
-      <c r="T5" s="34" t="n">
+      <c r="U5" s="34" t="n">
         <v>-0.2132075</v>
       </c>
-      <c r="U5" s="34" t="n">
+      <c r="V5" s="34" t="n">
         <v>-0.2785467</v>
       </c>
-      <c r="V5" s="34" t="n">
+      <c r="W5" s="34" t="n">
         <v>-0.5162413</v>
       </c>
     </row>
@@ -15182,19 +15188,24 @@
       <c r="Q6" s="39" t="n">
         <v>27.8</v>
       </c>
-      <c r="R6" s="41" t="n">
+      <c r="R6" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S6" s="41" t="n">
         <v>-0.175089</v>
       </c>
-      <c r="S6" s="41" t="n">
+      <c r="T6" s="41" t="n">
         <v>-0.2584773</v>
       </c>
-      <c r="T6" s="41" t="n">
+      <c r="U6" s="41" t="n">
         <v>-0.1246224</v>
       </c>
-      <c r="U6" s="41" t="n">
+      <c r="V6" s="41" t="n">
         <v>0.5515395000000001</v>
       </c>
-      <c r="V6" s="41" t="n">
+      <c r="W6" s="41" t="n">
         <v>0.6097222</v>
       </c>
     </row>
@@ -15256,19 +15267,24 @@
       <c r="Q7" s="39" t="n">
         <v>14.8</v>
       </c>
-      <c r="R7" s="34" t="n">
+      <c r="R7" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S7" s="34" t="n">
         <v>-0.1135492</v>
       </c>
-      <c r="S7" s="34" t="n">
+      <c r="T7" s="34" t="n">
         <v>-0.07315100000000001</v>
       </c>
-      <c r="T7" s="34" t="n">
+      <c r="U7" s="34" t="n">
         <v>0.2044332</v>
       </c>
-      <c r="U7" s="34" t="n">
+      <c r="V7" s="34" t="n">
         <v>0.0212626</v>
       </c>
-      <c r="V7" s="34" t="n">
+      <c r="W7" s="34" t="n">
         <v>0.1612072</v>
       </c>
     </row>
@@ -15330,19 +15346,24 @@
       <c r="Q8" s="39" t="n">
         <v>27.6</v>
       </c>
-      <c r="R8" s="41" t="n">
+      <c r="R8" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S8" s="41" t="n">
         <v>-0.1526151</v>
       </c>
-      <c r="S8" s="41" t="n">
+      <c r="T8" s="41" t="n">
         <v>-0.3488302</v>
       </c>
-      <c r="T8" s="41" t="n">
+      <c r="U8" s="41" t="n">
         <v>0.039751</v>
       </c>
-      <c r="U8" s="41" t="n">
+      <c r="V8" s="41" t="n">
         <v>0.8780277</v>
       </c>
-      <c r="V8" s="41" t="n">
+      <c r="W8" s="41" t="n">
         <v>0.4829235</v>
       </c>
     </row>
@@ -15404,19 +15425,24 @@
       <c r="Q9" s="39" t="n">
         <v>13.8</v>
       </c>
-      <c r="R9" s="34" t="n">
+      <c r="R9" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S9" s="34" t="n">
         <v>-0.0546512</v>
       </c>
-      <c r="S9" s="34" t="n">
+      <c r="T9" s="34" t="n">
         <v>0.101626</v>
       </c>
-      <c r="T9" s="34" t="n">
+      <c r="U9" s="34" t="n">
         <v>-0.151357</v>
       </c>
-      <c r="U9" s="34" t="n">
+      <c r="V9" s="34" t="n">
         <v>-0.4761598</v>
       </c>
-      <c r="V9" s="34" t="n">
+      <c r="W9" s="34" t="n">
         <v>-0.2930435</v>
       </c>
     </row>
@@ -15478,19 +15504,24 @@
       <c r="Q10" s="45" t="n">
         <v>43.6</v>
       </c>
-      <c r="R10" s="41" t="n">
+      <c r="R10" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S10" s="41" t="n">
         <v>-0.0071860914</v>
       </c>
-      <c r="S10" s="41" t="n">
+      <c r="T10" s="41" t="n">
         <v>-0.2177372</v>
       </c>
-      <c r="T10" s="41" t="n">
+      <c r="U10" s="41" t="n">
         <v>0.1933746</v>
       </c>
-      <c r="U10" s="41" t="n">
+      <c r="V10" s="41" t="n">
         <v>0.2285578</v>
       </c>
-      <c r="V10" s="41" t="n">
+      <c r="W10" s="41" t="n">
         <v>0.9443127</v>
       </c>
     </row>
@@ -15552,19 +15583,24 @@
       <c r="Q11" s="39" t="n">
         <v>11.3</v>
       </c>
-      <c r="R11" s="34" t="n">
+      <c r="R11" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S11" s="34" t="n">
         <v>-0.1063652</v>
       </c>
-      <c r="S11" s="34" t="n">
+      <c r="T11" s="34" t="n">
         <v>-0.2061012</v>
       </c>
-      <c r="T11" s="34" t="n">
+      <c r="U11" s="34" t="n">
         <v>-0.0557522</v>
       </c>
-      <c r="U11" s="34" t="n">
+      <c r="V11" s="34" t="n">
         <v>-0.0895904</v>
       </c>
-      <c r="V11" s="34" t="n">
+      <c r="W11" s="34" t="n">
         <v>0.1184486</v>
       </c>
     </row>
@@ -15626,19 +15662,24 @@
       <c r="Q12" s="39" t="n">
         <v>6.1</v>
       </c>
-      <c r="R12" s="41" t="n">
+      <c r="R12" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S12" s="41" t="n">
         <v>-0.0272109</v>
       </c>
-      <c r="S12" s="41" t="n">
+      <c r="T12" s="41" t="n">
         <v>-0.0793991</v>
       </c>
-      <c r="T12" s="41" t="n">
+      <c r="U12" s="41" t="n">
         <v>-0.3254717</v>
       </c>
-      <c r="U12" s="41" t="n">
+      <c r="V12" s="41" t="n">
         <v>-0.3035714</v>
       </c>
-      <c r="V12" s="41" t="n">
+      <c r="W12" s="41" t="n">
         <v>-0.3035714</v>
       </c>
     </row>
@@ -15700,19 +15741,24 @@
       <c r="Q13" s="39" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="R13" s="34" t="n">
+      <c r="R13" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S13" s="34" t="n">
         <v>-0.1748072</v>
       </c>
-      <c r="S13" s="34" t="n">
+      <c r="T13" s="34" t="n">
         <v>-0.4729064000000001</v>
       </c>
-      <c r="T13" s="34" t="n">
+      <c r="U13" s="34" t="n">
         <v>0.07718120000000001</v>
       </c>
-      <c r="U13" s="34" t="n">
+      <c r="V13" s="34" t="n">
         <v>-0.3502024</v>
       </c>
-      <c r="V13" s="34" t="n">
+      <c r="W13" s="34" t="n">
         <v>-0.5143722000000001</v>
       </c>
     </row>
@@ -15774,19 +15820,24 @@
       <c r="Q14" s="39" t="n">
         <v>17.6</v>
       </c>
-      <c r="R14" s="41" t="n">
+      <c r="R14" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S14" s="41" t="n">
         <v>-0.05880080000000001</v>
       </c>
-      <c r="S14" s="41" t="n">
+      <c r="T14" s="41" t="n">
         <v>-0.0897213</v>
       </c>
-      <c r="T14" s="41" t="n">
+      <c r="U14" s="41" t="n">
         <v>-0.1400188</v>
       </c>
-      <c r="U14" s="41" t="n">
+      <c r="V14" s="41" t="n">
         <v>-0.0193055</v>
       </c>
-      <c r="V14" s="41" t="n">
+      <c r="W14" s="41" t="n">
         <v>0.0590705</v>
       </c>
     </row>
@@ -15817,6 +15868,7 @@
       <c r="T17" s="17" t="n"/>
       <c r="U17" s="17" t="n"/>
       <c r="V17" s="17" t="n"/>
+      <c r="W17" s="17" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="18" t="inlineStr">
@@ -16256,9 +16308,9 @@
   <mergeCells count="3">
     <mergeCell ref="A2:V2"/>
     <mergeCell ref="A1:V1"/>
-    <mergeCell ref="A17:V17"/>
+    <mergeCell ref="A17:W17"/>
   </mergeCells>
-  <conditionalFormatting sqref="K5:K14">
+  <conditionalFormatting sqref="L5:L14">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -16270,7 +16322,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L5:L14">
+  <conditionalFormatting sqref="M5:M14">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -16282,7 +16334,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M14">
+  <conditionalFormatting sqref="N5:N14">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -16294,7 +16346,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N5:N14">
+  <conditionalFormatting sqref="O5:O14">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -16306,7 +16358,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P5:P14">
+  <conditionalFormatting sqref="Q5:Q14">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -16356,15 +16408,15 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R5:R14">
+  <conditionalFormatting sqref="K5:K14">
     <cfRule type="colorScale" priority="10">
       <colorScale>
-        <cfvo type="min"/>
         <cfvo type="num" val="0"/>
-        <cfvo type="max"/>
-        <color rgb="00E76F51"/>
-        <color rgb="00FFFFFF"/>
-        <color rgb="002A9D8F"/>
+        <cfvo type="num" val="50"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="00C1121F"/>
+        <color rgb="00F9C74F"/>
+        <color rgb="001A6B3C"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -16416,8 +16468,20 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="W5:W14">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="00E76F51"/>
+        <color rgb="00FFFFFF"/>
+        <color rgb="002A9D8F"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B19:B28">
-    <cfRule type="colorScale" priority="15">
+    <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="50"/>
@@ -16429,7 +16493,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C19:C28">
-    <cfRule type="colorScale" priority="16">
+    <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="50"/>
@@ -16441,7 +16505,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D19:D28">
-    <cfRule type="colorScale" priority="17">
+    <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="50"/>
@@ -16453,7 +16517,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E19:E28">
-    <cfRule type="colorScale" priority="18">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="50"/>
@@ -16465,7 +16529,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F19:F28">
-    <cfRule type="colorScale" priority="19">
+    <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="50"/>
@@ -16505,15 +16569,16 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -16748,19 +16813,24 @@
       <c r="Q5" s="39" t="n">
         <v>31.8</v>
       </c>
-      <c r="R5" s="34" t="n">
+      <c r="R5" s="23" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S5" s="34" t="n">
         <v>-0.0764</v>
       </c>
-      <c r="S5" s="34" t="n">
+      <c r="T5" s="34" t="n">
         <v>-0.1028425</v>
       </c>
-      <c r="T5" s="34" t="n">
+      <c r="U5" s="34" t="n">
         <v>-0.0592352</v>
       </c>
-      <c r="U5" s="34" t="n">
+      <c r="V5" s="34" t="n">
         <v>0.333465</v>
       </c>
-      <c r="V5" s="34" t="n">
+      <c r="W5" s="34" t="n">
         <v>0.4888348</v>
       </c>
     </row>
@@ -16822,19 +16892,24 @@
       <c r="Q6" s="45" t="n">
         <v>65.90000000000001</v>
       </c>
-      <c r="R6" s="41" t="n">
+      <c r="R6" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S6" s="41" t="n">
         <v>-0.1993195</v>
       </c>
-      <c r="S6" s="41" t="n">
+      <c r="T6" s="41" t="n">
         <v>-0.0620936</v>
       </c>
-      <c r="T6" s="41" t="n">
+      <c r="U6" s="41" t="n">
         <v>0.09556480000000001</v>
       </c>
-      <c r="U6" s="41" t="n">
+      <c r="V6" s="41" t="n">
         <v>0.3921843</v>
       </c>
-      <c r="V6" s="41" t="n">
+      <c r="W6" s="41" t="n">
         <v>0.8711027</v>
       </c>
     </row>
@@ -16896,19 +16971,24 @@
       <c r="Q7" s="39" t="n">
         <v>7.5</v>
       </c>
-      <c r="R7" s="34" t="n">
+      <c r="R7" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S7" s="34" t="n">
         <v>-0.009964050300000001</v>
       </c>
-      <c r="S7" s="34" t="n">
+      <c r="T7" s="34" t="n">
         <v>-0.1380438</v>
       </c>
-      <c r="T7" s="34" t="n">
+      <c r="U7" s="34" t="n">
         <v>-0.0779185</v>
       </c>
-      <c r="U7" s="34" t="n">
+      <c r="V7" s="34" t="n">
         <v>0.0477933</v>
       </c>
-      <c r="V7" s="34" t="n">
+      <c r="W7" s="34" t="n">
         <v>-0.0251504</v>
       </c>
     </row>
@@ -16970,19 +17050,24 @@
       <c r="Q8" s="39" t="n">
         <v>21.9</v>
       </c>
-      <c r="R8" s="41" t="n">
+      <c r="R8" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S8" s="41" t="n">
         <v>-0.2711404</v>
       </c>
-      <c r="S8" s="41" t="n">
+      <c r="T8" s="41" t="n">
         <v>-0.3827201</v>
       </c>
-      <c r="T8" s="41" t="n">
+      <c r="U8" s="41" t="n">
         <v>0.4733403</v>
       </c>
-      <c r="U8" s="41" t="n">
+      <c r="V8" s="41" t="n">
         <v>0.3097119</v>
       </c>
-      <c r="V8" s="41" t="n">
+      <c r="W8" s="41" t="n">
         <v>0.2127797</v>
       </c>
     </row>
@@ -17044,19 +17129,24 @@
       <c r="Q9" s="45" t="n">
         <v>60.3</v>
       </c>
-      <c r="R9" s="34" t="n">
+      <c r="R9" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S9" s="34" t="n">
         <v>-0.04738299999999999</v>
       </c>
-      <c r="S9" s="34" t="n">
+      <c r="T9" s="34" t="n">
         <v>-0.4553184</v>
       </c>
-      <c r="T9" s="34" t="n">
+      <c r="U9" s="34" t="n">
         <v>0.5034514</v>
       </c>
-      <c r="U9" s="34" t="n">
+      <c r="V9" s="34" t="n">
         <v>0.6971429</v>
       </c>
-      <c r="V9" s="34" t="n">
+      <c r="W9" s="34" t="n">
         <v>1.1809079</v>
       </c>
     </row>
@@ -17118,19 +17208,24 @@
       <c r="Q10" s="45" t="n">
         <v>41.2</v>
       </c>
-      <c r="R10" s="41" t="n">
+      <c r="R10" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S10" s="41" t="n">
         <v>0.3156425</v>
       </c>
-      <c r="S10" s="41" t="n">
+      <c r="T10" s="41" t="n">
         <v>0.369186</v>
       </c>
-      <c r="T10" s="41" t="n">
+      <c r="U10" s="41" t="n">
         <v>0.5292208</v>
       </c>
-      <c r="U10" s="41" t="n">
+      <c r="V10" s="41" t="n">
         <v>0.4101796</v>
       </c>
-      <c r="V10" s="41" t="n">
+      <c r="W10" s="41" t="n">
         <v>0.1432039</v>
       </c>
     </row>
@@ -17192,19 +17287,24 @@
       <c r="Q11" s="39" t="n">
         <v>2.3</v>
       </c>
-      <c r="R11" s="34" t="n">
+      <c r="R11" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S11" s="34" t="n">
         <v>-0.1703263</v>
       </c>
-      <c r="S11" s="34" t="n">
+      <c r="T11" s="34" t="n">
         <v>-0.126134</v>
       </c>
-      <c r="T11" s="34" t="n">
+      <c r="U11" s="34" t="n">
         <v>0.0011614173</v>
       </c>
-      <c r="U11" s="34" t="n">
+      <c r="V11" s="34" t="n">
         <v>-0.2896788</v>
       </c>
-      <c r="V11" s="34" t="n">
+      <c r="W11" s="34" t="n">
         <v>-0.3850181</v>
       </c>
     </row>
@@ -17266,19 +17366,24 @@
       <c r="Q12" s="39" t="n">
         <v>1.9</v>
       </c>
-      <c r="R12" s="41" t="n">
+      <c r="R12" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S12" s="41" t="n">
         <v>-0.003968254</v>
       </c>
-      <c r="S12" s="41" t="n">
+      <c r="T12" s="41" t="n">
         <v>-0.5299625</v>
       </c>
-      <c r="T12" s="41" t="n">
+      <c r="U12" s="41" t="n">
         <v>-0.2148071</v>
       </c>
-      <c r="U12" s="41" t="n">
+      <c r="V12" s="41" t="n">
         <v>-0.1334868</v>
       </c>
-      <c r="V12" s="41" t="n">
+      <c r="W12" s="41" t="n">
         <v>-0.2617647</v>
       </c>
     </row>
@@ -17340,19 +17445,24 @@
       <c r="Q13" s="39" t="n">
         <v>28</v>
       </c>
-      <c r="R13" s="34" t="n">
+      <c r="R13" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S13" s="34" t="n">
         <v>-0.07517310000000001</v>
       </c>
-      <c r="S13" s="34" t="n">
+      <c r="T13" s="34" t="n">
         <v>0.5008026</v>
       </c>
-      <c r="T13" s="34" t="n">
+      <c r="U13" s="34" t="n">
         <v>0.1150865</v>
       </c>
-      <c r="U13" s="34" t="n">
+      <c r="V13" s="34" t="n">
         <v>0.08405799999999999</v>
       </c>
-      <c r="V13" s="34" t="n">
+      <c r="W13" s="34" t="n">
         <v>0.2541918</v>
       </c>
     </row>
@@ -17414,19 +17524,24 @@
       <c r="Q14" s="39" t="n">
         <v>20</v>
       </c>
-      <c r="R14" s="41" t="n">
+      <c r="R14" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S14" s="41" t="n">
         <v>0.0315871</v>
       </c>
-      <c r="S14" s="41" t="n">
+      <c r="T14" s="41" t="n">
         <v>0.1158333</v>
       </c>
-      <c r="T14" s="41" t="n">
+      <c r="U14" s="41" t="n">
         <v>0.1047855</v>
       </c>
-      <c r="U14" s="41" t="n">
+      <c r="V14" s="41" t="n">
         <v>0.2239488</v>
       </c>
-      <c r="V14" s="41" t="n">
+      <c r="W14" s="41" t="n">
         <v>0.0939542</v>
       </c>
     </row>
@@ -17457,6 +17572,7 @@
       <c r="T17" s="17" t="n"/>
       <c r="U17" s="17" t="n"/>
       <c r="V17" s="17" t="n"/>
+      <c r="W17" s="17" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="18" t="inlineStr">
@@ -17896,9 +18012,9 @@
   <mergeCells count="3">
     <mergeCell ref="A2:V2"/>
     <mergeCell ref="A1:V1"/>
-    <mergeCell ref="A17:V17"/>
+    <mergeCell ref="A17:W17"/>
   </mergeCells>
-  <conditionalFormatting sqref="K5:K14">
+  <conditionalFormatting sqref="L5:L14">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -17910,7 +18026,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L5:L14">
+  <conditionalFormatting sqref="M5:M14">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -17922,7 +18038,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M14">
+  <conditionalFormatting sqref="N5:N14">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -17934,7 +18050,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N5:N14">
+  <conditionalFormatting sqref="O5:O14">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -17946,7 +18062,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P5:P14">
+  <conditionalFormatting sqref="Q5:Q14">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -17996,15 +18112,15 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R5:R14">
+  <conditionalFormatting sqref="K5:K14">
     <cfRule type="colorScale" priority="10">
       <colorScale>
-        <cfvo type="min"/>
         <cfvo type="num" val="0"/>
-        <cfvo type="max"/>
-        <color rgb="00E76F51"/>
-        <color rgb="00FFFFFF"/>
-        <color rgb="002A9D8F"/>
+        <cfvo type="num" val="50"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="00C1121F"/>
+        <color rgb="00F9C74F"/>
+        <color rgb="001A6B3C"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -18056,8 +18172,20 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="W5:W14">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="00E76F51"/>
+        <color rgb="00FFFFFF"/>
+        <color rgb="002A9D8F"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B19:B28">
-    <cfRule type="colorScale" priority="15">
+    <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="50"/>
@@ -18069,7 +18197,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C19:C28">
-    <cfRule type="colorScale" priority="16">
+    <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="50"/>
@@ -18081,7 +18209,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D19:D28">
-    <cfRule type="colorScale" priority="17">
+    <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="50"/>
@@ -18093,7 +18221,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E19:E28">
-    <cfRule type="colorScale" priority="18">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="50"/>
@@ -18105,7 +18233,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F19:F28">
-    <cfRule type="colorScale" priority="19">
+    <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="50"/>
@@ -18145,15 +18273,16 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -18388,19 +18517,24 @@
       <c r="Q5" s="39" t="n">
         <v>12.8</v>
       </c>
-      <c r="R5" s="34" t="n">
+      <c r="R5" s="23" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S5" s="34" t="n">
         <v>0.0141262</v>
       </c>
-      <c r="S5" s="34" t="n">
+      <c r="T5" s="34" t="n">
         <v>-0.0931133</v>
       </c>
-      <c r="T5" s="34" t="n">
+      <c r="U5" s="34" t="n">
         <v>-0.0975264</v>
       </c>
-      <c r="U5" s="34" t="n">
+      <c r="V5" s="34" t="n">
         <v>0.05274359999999999</v>
       </c>
-      <c r="V5" s="34" t="n">
+      <c r="W5" s="34" t="n">
         <v>-0.04320719999999999</v>
       </c>
     </row>
@@ -18462,19 +18596,24 @@
       <c r="Q6" s="39" t="n">
         <v>1.3</v>
       </c>
-      <c r="R6" s="41" t="n">
+      <c r="R6" s="23" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="S6" s="41" t="n">
         <v>-0.0709584</v>
       </c>
-      <c r="S6" s="41" t="n">
+      <c r="T6" s="41" t="n">
         <v>-0.0535139</v>
       </c>
-      <c r="T6" s="41" t="n">
+      <c r="U6" s="41" t="n">
         <v>-0.3008718</v>
       </c>
-      <c r="U6" s="41" t="n">
+      <c r="V6" s="41" t="n">
         <v>-0.3333648</v>
       </c>
-      <c r="V6" s="41" t="n">
+      <c r="W6" s="41" t="n">
         <v>-0.4225041</v>
       </c>
     </row>
@@ -18536,19 +18675,24 @@
       <c r="Q7" s="45" t="n">
         <v>51.1</v>
       </c>
-      <c r="R7" s="34" t="n">
+      <c r="R7" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S7" s="34" t="n">
         <v>-0.0364896</v>
       </c>
-      <c r="S7" s="34" t="n">
+      <c r="T7" s="34" t="n">
         <v>-0.1378796</v>
       </c>
-      <c r="T7" s="34" t="n">
+      <c r="U7" s="34" t="n">
         <v>0.3688928</v>
       </c>
-      <c r="U7" s="34" t="n">
+      <c r="V7" s="34" t="n">
         <v>0.5768058</v>
       </c>
-      <c r="V7" s="34" t="n">
+      <c r="W7" s="34" t="n">
         <v>0.7696747</v>
       </c>
     </row>
@@ -18610,19 +18754,24 @@
       <c r="Q8" s="39" t="n">
         <v>20.7</v>
       </c>
-      <c r="R8" s="41" t="n">
+      <c r="R8" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S8" s="41" t="n">
         <v>-0.0709867</v>
       </c>
-      <c r="S8" s="41" t="n">
+      <c r="T8" s="41" t="n">
         <v>0.09085499999999999</v>
       </c>
-      <c r="T8" s="41" t="n">
+      <c r="U8" s="41" t="n">
         <v>0.032458</v>
       </c>
-      <c r="U8" s="41" t="n">
+      <c r="V8" s="41" t="n">
         <v>0.0332732</v>
       </c>
-      <c r="V8" s="41" t="n">
+      <c r="W8" s="41" t="n">
         <v>0.1276465</v>
       </c>
     </row>
@@ -18684,19 +18833,24 @@
       <c r="Q9" s="39" t="n">
         <v>18.1</v>
       </c>
-      <c r="R9" s="34" t="n">
+      <c r="R9" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S9" s="34" t="n">
         <v>-0.0535698</v>
       </c>
-      <c r="S9" s="34" t="n">
+      <c r="T9" s="34" t="n">
         <v>0.04776</v>
       </c>
-      <c r="T9" s="34" t="n">
+      <c r="U9" s="34" t="n">
         <v>-0.09756930000000001</v>
       </c>
-      <c r="U9" s="34" t="n">
+      <c r="V9" s="34" t="n">
         <v>-0.0903795</v>
       </c>
-      <c r="V9" s="34" t="n">
+      <c r="W9" s="34" t="n">
         <v>-0.07589209999999999</v>
       </c>
     </row>
@@ -18758,19 +18912,24 @@
       <c r="Q10" s="39" t="n">
         <v>30.8</v>
       </c>
-      <c r="R10" s="41" t="n">
+      <c r="R10" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S10" s="41" t="n">
         <v>-0.0826219</v>
       </c>
-      <c r="S10" s="41" t="n">
+      <c r="T10" s="41" t="n">
         <v>-0.08009289999999999</v>
       </c>
-      <c r="T10" s="41" t="n">
+      <c r="U10" s="41" t="n">
         <v>0.0872921</v>
       </c>
-      <c r="U10" s="41" t="n">
+      <c r="V10" s="41" t="n">
         <v>0.1531466</v>
       </c>
-      <c r="V10" s="41" t="n">
+      <c r="W10" s="41" t="n">
         <v>0.3180873</v>
       </c>
     </row>
@@ -18832,19 +18991,24 @@
       <c r="Q11" s="45" t="n">
         <v>46.9</v>
       </c>
-      <c r="R11" s="34" t="n">
+      <c r="R11" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S11" s="34" t="n">
         <v>-0.0427199</v>
       </c>
-      <c r="S11" s="34" t="n">
+      <c r="T11" s="34" t="n">
         <v>0.1883114</v>
       </c>
-      <c r="T11" s="34" t="n">
+      <c r="U11" s="34" t="n">
         <v>0.001461039</v>
       </c>
-      <c r="U11" s="34" t="n">
+      <c r="V11" s="34" t="n">
         <v>0.1578236</v>
       </c>
-      <c r="V11" s="34" t="n">
+      <c r="W11" s="34" t="n">
         <v>0.301367</v>
       </c>
     </row>
@@ -18906,19 +19070,24 @@
       <c r="Q12" s="45" t="n">
         <v>48.8</v>
       </c>
-      <c r="R12" s="41" t="n">
+      <c r="R12" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S12" s="41" t="n">
         <v>-0.0492216</v>
       </c>
-      <c r="S12" s="41" t="n">
+      <c r="T12" s="41" t="n">
         <v>0.0507947</v>
       </c>
-      <c r="T12" s="41" t="n">
+      <c r="U12" s="41" t="n">
         <v>0.4366039</v>
       </c>
-      <c r="U12" s="41" t="n">
+      <c r="V12" s="41" t="n">
         <v>0.2596739</v>
       </c>
-      <c r="V12" s="41" t="n">
+      <c r="W12" s="41" t="n">
         <v>0.5150012</v>
       </c>
     </row>
@@ -18980,19 +19149,24 @@
       <c r="Q13" s="39" t="n">
         <v>23.5</v>
       </c>
-      <c r="R13" s="34" t="n">
+      <c r="R13" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S13" s="34" t="n">
         <v>-0.0783015</v>
       </c>
-      <c r="S13" s="34" t="n">
+      <c r="T13" s="34" t="n">
         <v>0.1319464</v>
       </c>
-      <c r="T13" s="34" t="n">
+      <c r="U13" s="34" t="n">
         <v>0.0026208026</v>
       </c>
-      <c r="U13" s="34" t="n">
+      <c r="V13" s="34" t="n">
         <v>0.0503647</v>
       </c>
-      <c r="V13" s="34" t="n">
+      <c r="W13" s="34" t="n">
         <v>-0.06054789999999999</v>
       </c>
     </row>
@@ -19054,19 +19228,24 @@
       <c r="Q14" s="39" t="n">
         <v>5.9</v>
       </c>
-      <c r="R14" s="41" t="n">
+      <c r="R14" s="27" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
+      <c r="S14" s="41" t="n">
         <v>-0.09878740000000001</v>
       </c>
-      <c r="S14" s="41" t="n">
+      <c r="T14" s="41" t="n">
         <v>0.0929931</v>
       </c>
-      <c r="T14" s="41" t="n">
+      <c r="U14" s="41" t="n">
         <v>-0.0420773</v>
       </c>
-      <c r="U14" s="41" t="n">
+      <c r="V14" s="41" t="n">
         <v>-0.5242846</v>
       </c>
-      <c r="V14" s="41" t="n">
+      <c r="W14" s="41" t="n">
         <v>-0.6187387</v>
       </c>
     </row>
@@ -19097,6 +19276,7 @@
       <c r="T17" s="17" t="n"/>
       <c r="U17" s="17" t="n"/>
       <c r="V17" s="17" t="n"/>
+      <c r="W17" s="17" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="18" t="inlineStr">
@@ -19536,9 +19716,9 @@
   <mergeCells count="3">
     <mergeCell ref="A2:V2"/>
     <mergeCell ref="A1:V1"/>
-    <mergeCell ref="A17:V17"/>
+    <mergeCell ref="A17:W17"/>
   </mergeCells>
-  <conditionalFormatting sqref="K5:K14">
+  <conditionalFormatting sqref="L5:L14">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -19550,7 +19730,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L5:L14">
+  <conditionalFormatting sqref="M5:M14">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -19562,7 +19742,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M14">
+  <conditionalFormatting sqref="N5:N14">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -19574,7 +19754,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N5:N14">
+  <conditionalFormatting sqref="O5:O14">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -19586,7 +19766,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P5:P14">
+  <conditionalFormatting sqref="Q5:Q14">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -19636,15 +19816,15 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R5:R14">
+  <conditionalFormatting sqref="K5:K14">
     <cfRule type="colorScale" priority="10">
       <colorScale>
-        <cfvo type="min"/>
         <cfvo type="num" val="0"/>
-        <cfvo type="max"/>
-        <color rgb="00E76F51"/>
-        <color rgb="00FFFFFF"/>
-        <color rgb="002A9D8F"/>
+        <cfvo type="num" val="50"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="00C1121F"/>
+        <color rgb="00F9C74F"/>
+        <color rgb="001A6B3C"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -19696,8 +19876,20 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="W5:W14">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="00E76F51"/>
+        <color rgb="00FFFFFF"/>
+        <color rgb="002A9D8F"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B19:B28">
-    <cfRule type="colorScale" priority="15">
+    <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="50"/>
@@ -19709,7 +19901,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C19:C28">
-    <cfRule type="colorScale" priority="16">
+    <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="50"/>
@@ -19721,7 +19913,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D19:D28">
-    <cfRule type="colorScale" priority="17">
+    <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="50"/>
@@ -19733,7 +19925,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E19:E28">
-    <cfRule type="colorScale" priority="18">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="50"/>
@@ -19745,7 +19937,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F19:F28">
-    <cfRule type="colorScale" priority="19">
+    <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="50"/>
@@ -19785,15 +19977,16 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">

</xml_diff>